<commit_message>
Brand PM attachments and rebuild cost tracker as multi-tab model
- Add Acqlerate branding (icon, wordmark, footer) to PM Approval RACI
  and Cost & Burn Rate Tracker templates
- Rebuild burn rate tracker into a 7-tab cost model: Rates (negotiated
  Fringe/OH/G&A/Fee), FundingMods (per-mod TOA log), Dashboard, Labor,
  ODCs, Travel, and Instructions
- Update finance-8 attachment entry to reference the new file
</commit_message>
<xml_diff>
--- a/client/public/examples/pm-approval-raci.xlsx
+++ b/client/public/examples/pm-approval-raci.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +59,36 @@
       <color rgb="001F3864"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="0001696F"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF01696F"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF0F172A"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -93,7 +123,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -115,11 +145,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -158,6 +232,13 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -232,6 +313,72 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="381000" cy="381000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="304800" cy="304800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -523,201 +670,216 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="105" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>Acqlerate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>DoD Acquisition Training  ·  acqlerate.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Contractor PM Approval Authority RACI — How to Use This</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>What this is for:</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>A quick-reference map of who actually has authority over the approvals a contractor PM deals with</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>day to day: invoices, travel, ODCs, subcontractor costs, timesheets, and more. New PMs often assume</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>"I approve it because I manage the program." Half of these, you don't. Knowing which half before</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>you sign something is what keeps you out of an unauthorized commitment.</t>
+          <t>A quick-reference map of who actually has authority over the approvals a contractor PM deals with</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>day to day: invoices, travel, ODCs, subcontractor costs, timesheets, and more. New PMs often assume</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>How to read a RACI:</t>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>"I approve it because I manage the program." Half of these, you don't. Knowing which half before</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  R = Responsible  — does the work / prepares the item</t>
+          <t>you sign something is what keeps you out of an unauthorized commitment.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  A = Accountable  — owns the decision, signs off, answers for it if it's wrong (exactly one A per row)</t>
-        </is>
-      </c>
+      <c r="A11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  C = Consulted    — gives input before the decision, two-way conversation</t>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>How to read a RACI:</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  I = Informed     — told after the fact, one-way notification</t>
+          <t xml:space="preserve">  R = Responsible  — does the work / prepares the item</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A = Accountable  — owns the decision, signs off, answers for it if it's wrong (exactly one A per row)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>The roles across the top are generic — swap in your own company's titles if they differ. The point</t>
+          <t xml:space="preserve">  C = Consulted    — gives input before the decision, two-way conversation</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>isn't the exact labels, it's the pattern: on nearly every row, the PM is Responsible or Consulted,</t>
+          <t xml:space="preserve">  I = Informed     — told after the fact, one-way notification</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>almost never Accountable for anything involving government money. That authority sits with your</t>
-        </is>
-      </c>
+      <c r="A17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Contracts/Finance function on your side, and with the CO on the government side. Mixing that up is</t>
+          <t>The roles across the top are generic — swap in your own company's titles if they differ. The point</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>exactly how PMs end up making commitments they don't have the authority to make.</t>
+          <t>isn't the exact labels, it's the pattern: on nearly every row, the PM is Responsible or Consulted,</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>almost never Accountable for anything involving government money. That authority sits with your</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>This reflects common practice on cost-reimbursable and T&amp;M federal services contracts. Your specific</t>
+          <t>Contracts/Finance function on your side, and with the CO on the government side. Mixing that up is</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>exactly how PMs end up making commitments they don't have the authority to make.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>This reflects common practice on cost-reimbursable and T&amp;M federal services contracts. Your specific</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>contract, your company's delegation of authority policy, and your accounting system's controls are</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>what actually govern — check those before you rely on this for a real approval decision.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>One exception to "one A per row":</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Two rows ("Consent to subcontract" and "Approve out-of-scope work a COR requests") show</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>two A's on purpose. Those decisions cross the contractor/government line — your Contracts</t>
+          <t>what actually govern — check those before you rely on this for a real approval decision.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Manager is Accountable for your company saying yes, AND the CO is separately Accountable for</t>
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>One exception to "one A per row":</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>the government saying yes. Both have to sign off independently. Collapsing that to one A would hide</t>
+          <t>Two rows ("Consent to subcontract" and "Approve out-of-scope work a COR requests") show</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t>two A's on purpose. Those decisions cross the contractor/government line — your Contracts</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Manager is Accountable for your company saying yes, AND the CO is separately Accountable for</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>the government saying yes. Both have to sign off independently. Collapsing that to one A would hide</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
           <t>the exact thing this tool exists to show you.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -727,7 +889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -740,198 +902,87 @@
     <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="B1" s="19" t="inlineStr">
+        <is>
+          <t>Acqlerate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="20" t="inlineStr">
+        <is>
+          <t>The DoD Acquisitions Learning Platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Contractor PM Approval Authority — RACI Matrix</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Who actually decides — not just who touches the paperwork</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+    <row r="6" ht="30" customHeight="1"/>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Approval / Decision</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Program
 Manager (PM)</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Subcontracts /
 Procurement</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Finance / Cost
 Analyst</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Contracts
 Manager (Prime)</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Government
 COR</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Contracting
 Officer (CO)</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Approve employee timesheet / labor charge</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Labor &amp; Timekeeping</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Approve overtime for a task</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Labor &amp; Timekeeping</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="H6" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Approve a labor category substitution (different person, same CLIN)</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Labor &amp; Timekeeping</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-    </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Approve Key Personnel substitution</t>
+          <t>Approve employee timesheet / labor charge</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -939,9 +990,9 @@
           <t>Labor &amp; Timekeeping</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -949,56 +1000,56 @@
           <t>I</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Approve a subcontractor invoice for payment</t>
+          <t>Approve overtime for a task</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Invoices &amp; Payments</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="inlineStr">
+          <t>Labor &amp; Timekeeping</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
@@ -1015,17 +1066,17 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Approve the prime's invoice to the government</t>
+          <t>Approve a labor category substitution (different person, same CLIN)</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Invoices &amp; Payments</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
+          <t>Labor &amp; Timekeeping</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>R</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -1033,9 +1084,9 @@
           <t>I</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -1043,26 +1094,26 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Approve an Other Direct Cost (ODC) purchase (materials, travel-related buys)</t>
+          <t>Approve Key Personnel substitution</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>ODCs</t>
+          <t>Labor &amp; Timekeeping</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
@@ -1070,41 +1121,41 @@
           <t>R</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Review / certify ODCs are allowable, allocable &amp; reasonable before billing</t>
+          <t>Approve a subcontractor invoice for payment</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>ODCs</t>
+          <t>Invoices &amp; Payments</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
@@ -1112,9 +1163,9 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>R</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -1122,9 +1173,9 @@
           <t>A</t>
         </is>
       </c>
-      <c r="F12" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
@@ -1141,17 +1192,17 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Approve an employee travel request</t>
+          <t>Approve the prime's invoice to the government</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Travel</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>Invoices &amp; Payments</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
@@ -1159,14 +1210,14 @@
           <t>I</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
@@ -1174,21 +1225,21 @@
           <t>I</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Approve travel that exceeds JTR/GSA per diem or requires an exception</t>
+          <t>Approve an Other Direct Cost (ODC) purchase (materials, travel-related buys)</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Travel</t>
+          <t>ODCs</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
@@ -1196,24 +1247,24 @@
           <t>R</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="E14" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
         </is>
       </c>
       <c r="H14" s="9" t="inlineStr">
@@ -1225,12 +1276,12 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Approve a subcontract purchase order / place a sub on contract</t>
+          <t>Review / certify ODCs are allowable, allocable &amp; reasonable before billing</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Subcontracting</t>
+          <t>ODCs</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
@@ -1238,19 +1289,19 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F15" s="11" t="inlineStr">
-        <is>
-          <t>R</t>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
@@ -1258,88 +1309,88 @@
           <t>I</t>
         </is>
       </c>
-      <c r="H15" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Consent to subcontract (above CO consent threshold)</t>
+          <t>Approve an employee travel request</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Subcontracting</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G16" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Approve a subcontractor rate increase (option year escalation)</t>
+          <t>Approve travel that exceeds JTR/GSA per diem or requires an exception</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Subcontracting</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="inlineStr">
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F17" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="H17" s="9" t="inlineStr">
@@ -1351,54 +1402,54 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Approve out-of-scope work a COR verbally requests</t>
+          <t>Approve a subcontract purchase order / place a sub on contract</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Scope &amp; Changes</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
+          <t>Subcontracting</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G18" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Approve a formal contract modification</t>
+          <t>Consent to subcontract (above CO consent threshold)</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Scope &amp; Changes</t>
+          <t>Subcontracting</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
@@ -1406,19 +1457,19 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
@@ -1435,32 +1486,32 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Sign / submit a Request for Equitable Adjustment (REA)</t>
+          <t>Approve a subcontractor rate increase (option year escalation)</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Scope &amp; Changes</t>
-        </is>
-      </c>
-      <c r="C20" s="11" t="inlineStr">
+          <t>Subcontracting</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
@@ -1477,12 +1528,12 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Approve the monthly Estimate to Complete (ETC) / EAC figure</t>
+          <t>Approve out-of-scope work a COR verbally requests</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Cost &amp; Budget</t>
+          <t>Scope &amp; Changes</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -1495,41 +1546,41 @@
           <t>I</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F21" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="G21" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="H21" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Approve drawing down Management Reserve</t>
+          <t>Approve a formal contract modification</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Cost &amp; Budget</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="inlineStr">
-        <is>
-          <t>R</t>
+          <t>Scope &amp; Changes</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
@@ -1537,9 +1588,9 @@
           <t>I</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
@@ -1547,26 +1598,26 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G22" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="H22" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Approve/submit the Monthly Status Report (MSR)</t>
+          <t>Sign / submit a Request for Equitable Adjustment (REA)</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Reporting</t>
+          <t>Scope &amp; Changes</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
@@ -1603,17 +1654,17 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Accept a CDRL deliverable as complete (government-side)</t>
+          <t>Approve the monthly Estimate to Complete (ETC) / EAC figure</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Deliverables</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
+          <t>Cost &amp; Budget</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>R</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
@@ -1621,41 +1672,41 @@
           <t>I</t>
         </is>
       </c>
-      <c r="E24" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="G24" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H24" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Certify an Incurred Cost Submission (ICS) to DCAA</t>
+          <t>Approve drawing down Management Reserve</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Compliance &amp; Audit</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
+          <t>Cost &amp; Budget</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>R</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
@@ -1663,14 +1714,14 @@
           <t>I</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
@@ -1687,109 +1738,230 @@
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
+          <t>Approve/submit the Monthly Status Report (MSR)</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Reporting</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Accept a CDRL deliverable as complete (government-side)</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Deliverables</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Certify an Incurred Cost Submission (ICS) to DCAA</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Compliance &amp; Audit</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
           <t>Respond to a DCAA records request</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>Compliance &amp; Audit</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
+      <c r="C29" s="21" t="n"/>
+      <c r="D29" s="21" t="n"/>
+      <c r="E29" s="22" t="n"/>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Legend:</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="E26" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="H26" s="10" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Legend:</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Responsible — does the work</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>Accountable — owns the decision (one per row)</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="14" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Consulted — input sought beforehand</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="15" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>Informed — notified after the fact</t>
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>Acqlerate  ·  DoD Acquisition Training  ·  acqlerate.com</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="4">
     <mergeCell ref="B31:E31"/>
-    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="B29:E29"/>
     <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="A1:H1"/>
     <mergeCell ref="B32:E32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>